<commit_message>
add new files and notes
</commit_message>
<xml_diff>
--- a/ABAP Programming/Select-Screen And Select-Query.xlsx
+++ b/ABAP Programming/Select-Screen And Select-Query.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ABAP 2026\ABAP Programming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D678A031-7CC1-4D96-8639-F88A2400EF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E3D1CC-F7C2-4597-9EF0-CCBD4681781F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4212" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Select-Screen Program Name </t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>zorder_no_hdr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SQL Program Name </t>
+  </si>
+  <si>
+    <t>ZSQLJOINS_SHUBHAM</t>
   </si>
 </sst>
 </file>
@@ -411,11 +417,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4:F8"/>
+  <dimension ref="B4:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -458,7 +464,16 @@
         <v>9</v>
       </c>
     </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>